<commit_message>
update schedule with titles
</commit_message>
<xml_diff>
--- a/RSI_2026_Schedule.xlsx
+++ b/RSI_2026_Schedule.xlsx
@@ -794,7 +794,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Characterizing Myo15-Cre Recombination in Cochlear Hair Cells to Validate Disease Models for Usher Syndrome Type 1F Gene Therapy​</t>
+          <t>Characterizing Myo15-Cre Recombination in Cochlear Hair Cells to Validate Disease Models for Usher Syndrome Type 1F Gene Therapy</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>(Title TBD)</t>
+          <t>Interactions of lipid droplets and Them1-containing condensates to regulate metabolism</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>(Title TBD)</t>
+          <t>Hybrid controls strategy for Automatic Laser Beam Alignment</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -4238,7 +4238,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>(Title TBD)</t>
+          <t>Critical Groups of Signed Subdivided Wheels</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">

</xml_diff>